<commit_message>
Shto lidhjen automatike me cTrader
cBot-i RaportiSync dërgon çdo trade të mbyllur (data, pair, setup, R:R
nga SL/TP fillestare, statusi, P/L real) te një Google Apps Script që e
shkruan si rresht të ri te fleta Raporti, pa dublikata. Raporti merr
kolonën e fshehur AC për ID-në e pozicionit dhe udhëzimet hap pas hapi.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016mxa5PvD4pus7Qj6wiPj4z
</commit_message>
<xml_diff>
--- a/Raporti_i_Analizave.xlsx
+++ b/Raporti_i_Analizave.xlsx
@@ -78,7 +78,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="91">
   <si>
     <t xml:space="preserve">RAPORTI I ANALIZAVE</t>
   </si>
@@ -135,6 +135,9 @@
   </si>
   <si>
     <t xml:space="preserve">Kategoria</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cTrader ID</t>
   </si>
   <si>
     <t xml:space="preserve">EUR/JPY</t>
@@ -336,6 +339,12 @@
   </si>
   <si>
     <t xml:space="preserve">Ngarkoje skedarin në Google Drive → hape me Google Sheets (ose: File → Import → Upload).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lidhja me cTrader</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trade-t mund të vijnë automatikisht nga cTrader: shih ctrader/UDHEZIME.md (cBot RaportiSync + Google Apps Script).</t>
   </si>
   <si>
     <t xml:space="preserve">Ngjyrat</t>
@@ -1294,11 +1303,11 @@
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:axId val="66572534"/>
-        <c:axId val="8607563"/>
+        <c:axId val="71630230"/>
+        <c:axId val="89389392"/>
       </c:areaChart>
       <c:catAx>
-        <c:axId val="66572534"/>
+        <c:axId val="71630230"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1330,14 +1339,14 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="8607563"/>
+        <c:crossAx val="89389392"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="8607563"/>
+        <c:axId val="89389392"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1376,7 +1385,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="66572534"/>
+        <c:crossAx val="71630230"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -1498,11 +1507,11 @@
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:axId val="80032504"/>
-        <c:axId val="97981801"/>
+        <c:axId val="82626296"/>
+        <c:axId val="54776767"/>
       </c:areaChart>
       <c:catAx>
-        <c:axId val="80032504"/>
+        <c:axId val="82626296"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1534,14 +1543,14 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="97981801"/>
+        <c:crossAx val="54776767"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="97981801"/>
+        <c:axId val="54776767"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1580,7 +1589,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="80032504"/>
+        <c:crossAx val="82626296"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -1883,7 +1892,7 @@
     <tabColor rgb="FF22C55E"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:AB514"/>
+  <dimension ref="A1:AC514"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="2"/>
@@ -1897,7 +1906,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="28"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="3"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="11" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="28" min="26" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="29" min="26" style="0" width="13"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="9.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2195,6 +2204,9 @@
       <c r="AB11" s="16" t="s">
         <v>18</v>
       </c>
+      <c r="AC11" s="16" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="1"/>
@@ -2202,16 +2214,16 @@
         <v>46029</v>
       </c>
       <c r="C12" s="18" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D12" s="18" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E12" s="19" t="n">
         <v>1.4</v>
       </c>
       <c r="F12" s="20" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G12" s="21" t="n">
         <f aca="false">IF($AB12="","",Cilësimet!$C$3*(INDEX(Cilësimet!$C$6:$C$10,MATCH($F12,Cilësimet!$A$6:$A$10,0))*N($E12)+INDEX(Cilësimet!$D$6:$D$10,MATCH($F12,Cilësimet!$A$6:$A$10,0))))</f>
@@ -2222,7 +2234,7 @@
         <v>0.00350000000000006</v>
       </c>
       <c r="I12" s="23" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="J12" s="1"/>
       <c r="K12" s="1"/>
@@ -2889,7 +2901,7 @@
       <c r="I29" s="23"/>
       <c r="J29" s="1"/>
       <c r="K29" s="25" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="L29" s="1"/>
       <c r="M29" s="1"/>
@@ -2930,7 +2942,7 @@
       <c r="I30" s="23"/>
       <c r="J30" s="1"/>
       <c r="K30" s="25" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="L30" s="1"/>
       <c r="M30" s="1"/>
@@ -21868,7 +21880,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="26" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -21894,7 +21906,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="27" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B3" s="1"/>
       <c r="C3" s="28" t="n">
@@ -21926,36 +21938,36 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="30" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B5" s="30" t="s">
         <v>18</v>
       </c>
       <c r="C5" s="30" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D5" s="30" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E5" s="1"/>
       <c r="F5" s="18" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G5" s="1"/>
       <c r="H5" s="18" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="I5" s="1"/>
       <c r="J5" s="31" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="32" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B6" s="18" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C6" s="19" t="n">
         <v>1</v>
@@ -21965,23 +21977,23 @@
       </c>
       <c r="E6" s="1"/>
       <c r="F6" s="18" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="G6" s="1"/>
       <c r="H6" s="18" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="I6" s="1"/>
       <c r="J6" s="25" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="33" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B7" s="18" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C7" s="19" t="n">
         <v>0.75</v>
@@ -21991,23 +22003,23 @@
       </c>
       <c r="E7" s="1"/>
       <c r="F7" s="18" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="G7" s="1"/>
       <c r="H7" s="18" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="I7" s="1"/>
       <c r="J7" s="25" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="34" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B8" s="18" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C8" s="19" t="n">
         <v>0.25</v>
@@ -22017,23 +22029,23 @@
       </c>
       <c r="E8" s="1"/>
       <c r="F8" s="18" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G8" s="1"/>
       <c r="H8" s="18" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="I8" s="1"/>
       <c r="J8" s="25" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="35" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B9" s="18" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C9" s="19" t="n">
         <v>0</v>
@@ -22043,23 +22055,23 @@
       </c>
       <c r="E9" s="1"/>
       <c r="F9" s="18" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="G9" s="1"/>
       <c r="H9" s="18" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="I9" s="1"/>
       <c r="J9" s="25" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="36" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B10" s="18" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C10" s="19" t="n">
         <v>0</v>
@@ -22069,15 +22081,15 @@
       </c>
       <c r="E10" s="1"/>
       <c r="F10" s="18" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="G10" s="1"/>
       <c r="H10" s="18" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="I10" s="1"/>
       <c r="J10" s="25" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22087,15 +22099,15 @@
       <c r="D11" s="1"/>
       <c r="E11" s="1"/>
       <c r="F11" s="18" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="G11" s="1"/>
       <c r="H11" s="18" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="I11" s="1"/>
       <c r="J11" s="25" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22105,20 +22117,20 @@
       <c r="D12" s="1"/>
       <c r="E12" s="1"/>
       <c r="F12" s="18" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G12" s="1"/>
       <c r="H12" s="18" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="I12" s="1"/>
       <c r="J12" s="25" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="25" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B13" s="1"/>
       <c r="C13" s="1"/>
@@ -22127,7 +22139,7 @@
       <c r="F13" s="1"/>
       <c r="G13" s="1"/>
       <c r="H13" s="18" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I13" s="1"/>
       <c r="J13" s="1"/>
@@ -22141,7 +22153,7 @@
       <c r="F14" s="1"/>
       <c r="G14" s="1"/>
       <c r="H14" s="18" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="I14" s="1"/>
       <c r="J14" s="1"/>
@@ -22155,7 +22167,7 @@
       <c r="F15" s="1"/>
       <c r="G15" s="1"/>
       <c r="H15" s="18" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="I15" s="1"/>
       <c r="J15" s="1"/>
@@ -22169,7 +22181,7 @@
       <c r="F16" s="1"/>
       <c r="G16" s="1"/>
       <c r="H16" s="18" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="I16" s="1"/>
       <c r="J16" s="1"/>
@@ -22183,7 +22195,7 @@
       <c r="F17" s="1"/>
       <c r="G17" s="1"/>
       <c r="H17" s="18" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="I17" s="1"/>
       <c r="J17" s="1"/>
@@ -22197,7 +22209,7 @@
       <c r="F18" s="1"/>
       <c r="G18" s="1"/>
       <c r="H18" s="18" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="I18" s="1"/>
       <c r="J18" s="1"/>
@@ -22211,7 +22223,7 @@
       <c r="F19" s="1"/>
       <c r="G19" s="1"/>
       <c r="H19" s="18" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="I19" s="1"/>
       <c r="J19" s="1"/>
@@ -22225,7 +22237,7 @@
       <c r="F20" s="1"/>
       <c r="G20" s="1"/>
       <c r="H20" s="18" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I20" s="1"/>
       <c r="J20" s="1"/>
@@ -22239,7 +22251,7 @@
       <c r="F21" s="1"/>
       <c r="G21" s="1"/>
       <c r="H21" s="18" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="I21" s="1"/>
       <c r="J21" s="1"/>
@@ -22253,7 +22265,7 @@
       <c r="F22" s="1"/>
       <c r="G22" s="1"/>
       <c r="H22" s="18" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I22" s="1"/>
       <c r="J22" s="1"/>
@@ -22267,7 +22279,7 @@
       <c r="F23" s="1"/>
       <c r="G23" s="1"/>
       <c r="H23" s="18" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="I23" s="1"/>
       <c r="J23" s="1"/>
@@ -22281,7 +22293,7 @@
       <c r="F24" s="1"/>
       <c r="G24" s="1"/>
       <c r="H24" s="18" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="I24" s="1"/>
       <c r="J24" s="1"/>
@@ -22503,7 +22515,7 @@
     <row r="2" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="37"/>
       <c r="B2" s="38" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22513,43 +22525,43 @@
     <row r="4" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="37"/>
       <c r="B4" s="40" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="37"/>
       <c r="B5" s="39" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="37"/>
       <c r="B6" s="39" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="37"/>
       <c r="B7" s="39" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="37"/>
       <c r="B8" s="39" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="37"/>
       <c r="B9" s="39" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="37"/>
       <c r="B10" s="39" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22559,37 +22571,37 @@
     <row r="12" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="37"/>
       <c r="B12" s="40" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="37"/>
       <c r="B13" s="39" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="37"/>
       <c r="B14" s="39" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="37"/>
       <c r="B15" s="39" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="37"/>
       <c r="B16" s="39" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="37"/>
       <c r="B17" s="39" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22599,13 +22611,13 @@
     <row r="19" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="37"/>
       <c r="B19" s="40" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="37"/>
       <c r="B20" s="39" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22615,26 +22627,30 @@
     <row r="22" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="37"/>
       <c r="B22" s="40" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="37"/>
       <c r="B23" s="39" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="37"/>
-      <c r="B24" s="37"/>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B24" s="39"/>
+    </row>
+    <row r="25" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="37"/>
-      <c r="B25" s="37"/>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B25" s="40" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="37"/>
-      <c r="B26" s="37"/>
+      <c r="B26" s="39" t="s">
+        <v>90</v>
+      </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="37"/>

</xml_diff>